<commit_message>
chore: Backfill rubrics scores and priority tiers for all historical database rows
</commit_message>
<xml_diff>
--- a/News_Dashboard/data/raw_news_database_Mondee.xlsx
+++ b/News_Dashboard/data/raw_news_database_Mondee.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R17"/>
+  <dimension ref="A1:T17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -519,6 +519,16 @@
           <t>Target_Brand</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Criticality_Score</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Priority_Tier</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -609,6 +619,14 @@
           <t>Abhee, Mondee</t>
         </is>
       </c>
+      <c r="S2" t="n">
+        <v>3</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Tier 4 - Low</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -697,6 +715,14 @@
       <c r="R3" t="inlineStr">
         <is>
           <t>Mondee</t>
+        </is>
+      </c>
+      <c r="S3" t="n">
+        <v>10</v>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Tier 4 - Low</t>
         </is>
       </c>
     </row>
@@ -796,6 +822,14 @@
           <t>Abhee, Mondee</t>
         </is>
       </c>
+      <c r="S4" t="n">
+        <v>3</v>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Tier 4 - Low</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -886,6 +920,14 @@
           <t>Abhee, Mondee</t>
         </is>
       </c>
+      <c r="S5" t="n">
+        <v>3</v>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Tier 4 - Low</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -977,6 +1019,14 @@
       <c r="R6" t="inlineStr">
         <is>
           <t>Abhee, Mondee</t>
+        </is>
+      </c>
+      <c r="S6" t="n">
+        <v>3</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Tier 4 - Low</t>
         </is>
       </c>
     </row>
@@ -1074,6 +1124,14 @@
           <t>Abhee, Mondee</t>
         </is>
       </c>
+      <c r="S7" t="n">
+        <v>3</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Tier 4 - Low</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1167,6 +1225,14 @@
       <c r="R8" t="inlineStr">
         <is>
           <t>Abhee, Mondee</t>
+        </is>
+      </c>
+      <c r="S8" t="n">
+        <v>3</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Tier 4 - Low</t>
         </is>
       </c>
     </row>
@@ -1263,6 +1329,14 @@
       <c r="R9" t="inlineStr">
         <is>
           <t>Abhee, Mondee</t>
+        </is>
+      </c>
+      <c r="S9" t="n">
+        <v>3</v>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Tier 4 - Low</t>
         </is>
       </c>
     </row>
@@ -1386,6 +1460,14 @@
           <t>Abhee, Mondee</t>
         </is>
       </c>
+      <c r="S10" t="n">
+        <v>3</v>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Tier 4 - Low</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1492,6 +1574,14 @@
           <t>Abhee, Mondee</t>
         </is>
       </c>
+      <c r="S11" t="n">
+        <v>3</v>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Tier 4 - Low</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1589,6 +1679,14 @@
           <t>Abhee, Mondee</t>
         </is>
       </c>
+      <c r="S12" t="n">
+        <v>3</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>Tier 4 - Low</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1679,6 +1777,14 @@
           <t>Abhee, Mondee</t>
         </is>
       </c>
+      <c r="S13" t="n">
+        <v>3</v>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Tier 4 - Low</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1769,6 +1875,14 @@
           <t>Abhee, Mondee</t>
         </is>
       </c>
+      <c r="S14" t="n">
+        <v>3</v>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Tier 4 - Low</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1857,6 +1971,14 @@
       <c r="R15" t="inlineStr">
         <is>
           <t>Abhee, Mondee</t>
+        </is>
+      </c>
+      <c r="S15" t="n">
+        <v>3</v>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Tier 4 - Low</t>
         </is>
       </c>
     </row>
@@ -1961,6 +2083,14 @@
       <c r="R16" t="inlineStr">
         <is>
           <t>Mondee</t>
+        </is>
+      </c>
+      <c r="S16" t="n">
+        <v>13</v>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Tier 4 - Low</t>
         </is>
       </c>
     </row>
@@ -2082,6 +2212,14 @@
           <t>Mondee</t>
         </is>
       </c>
+      <c r="S17" t="n">
+        <v>13</v>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>Tier 4 - Low</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
made changes for rubrics and llm sentiment backfill
</commit_message>
<xml_diff>
--- a/News_Dashboard/data/raw_news_database_Mondee.xlsx
+++ b/News_Dashboard/data/raw_news_database_Mondee.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T20"/>
+  <dimension ref="A1:U20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -542,6 +542,11 @@
           <t>Priority_Tier</t>
         </is>
       </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>UI_Tab_Mapping</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -604,7 +609,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -633,11 +638,16 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
           <t>Tier 4 - Low</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Product</t>
         </is>
       </c>
     </row>
@@ -702,7 +712,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -731,11 +741,16 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
           <t>Tier 4 - Low</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Overview</t>
         </is>
       </c>
     </row>
@@ -836,11 +851,16 @@
         </is>
       </c>
       <c r="S4" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
           <t>Tier 4 - Low</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Product</t>
         </is>
       </c>
     </row>
@@ -905,7 +925,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -934,11 +954,16 @@
         </is>
       </c>
       <c r="S5" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
           <t>Tier 4 - Low</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Product</t>
         </is>
       </c>
     </row>
@@ -1035,11 +1060,16 @@
         </is>
       </c>
       <c r="S6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
           <t>Tier 4 - Low</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Overview</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1139,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1138,11 +1168,16 @@
         </is>
       </c>
       <c r="S7" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
           <t>Tier 4 - Low</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Product</t>
         </is>
       </c>
     </row>
@@ -1241,11 +1276,16 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
           <t>Tier 4 - Low</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Growth</t>
         </is>
       </c>
     </row>
@@ -1345,11 +1385,16 @@
         </is>
       </c>
       <c r="S9" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
           <t>Tier 4 - Low</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Product</t>
         </is>
       </c>
     </row>
@@ -1481,6 +1526,11 @@
           <t>Tier 4 - Low</t>
         </is>
       </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1588,11 +1638,16 @@
         </is>
       </c>
       <c r="S11" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>
           <t>Tier 4 - Low</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Product</t>
         </is>
       </c>
     </row>
@@ -1693,11 +1748,16 @@
         </is>
       </c>
       <c r="S12" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="T12" t="inlineStr">
         <is>
           <t>Tier 4 - Low</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Growth</t>
         </is>
       </c>
     </row>
@@ -1762,7 +1822,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1791,11 +1851,16 @@
         </is>
       </c>
       <c r="S13" t="n">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="T13" t="inlineStr">
         <is>
           <t>Tier 4 - Low</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Product</t>
         </is>
       </c>
     </row>
@@ -1860,7 +1925,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1889,11 +1954,16 @@
         </is>
       </c>
       <c r="S14" t="n">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="T14" t="inlineStr">
         <is>
           <t>Tier 4 - Low</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Product</t>
         </is>
       </c>
     </row>
@@ -1958,7 +2028,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1987,11 +2057,16 @@
         </is>
       </c>
       <c r="S15" t="n">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="T15" t="inlineStr">
         <is>
           <t>Tier 4 - Low</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Product</t>
         </is>
       </c>
     </row>
@@ -2070,7 +2145,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2099,11 +2174,16 @@
         </is>
       </c>
       <c r="S16" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="T16" t="inlineStr">
         <is>
           <t>Tier 4 - Low</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Overview</t>
         </is>
       </c>
     </row>
@@ -2226,11 +2306,16 @@
         </is>
       </c>
       <c r="S17" t="n">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="T17" t="inlineStr">
         <is>
           <t>Tier 4 - Low</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Product</t>
         </is>
       </c>
     </row>
@@ -2324,11 +2409,16 @@
         </is>
       </c>
       <c r="S18" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="T18" t="inlineStr">
         <is>
           <t>Tier 4 - Low</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>Overview</t>
         </is>
       </c>
     </row>
@@ -2422,11 +2512,16 @@
         </is>
       </c>
       <c r="S19" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="T19" t="inlineStr">
         <is>
           <t>Tier 4 - Low</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Overview</t>
         </is>
       </c>
     </row>
@@ -2520,11 +2615,16 @@
         </is>
       </c>
       <c r="S20" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="T20" t="inlineStr">
         <is>
           <t>Tier 4 - Low</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>Product</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement dynamic synthesized CEO insights generated on backend and stored in Excel databases
</commit_message>
<xml_diff>
--- a/News_Dashboard/data/raw_news_database_Mondee.xlsx
+++ b/News_Dashboard/data/raw_news_database_Mondee.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw_News" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CEO_Insights" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Raw_News'!$A$1:$T$20</definedName>
@@ -2632,4 +2633,369 @@
   <autoFilter ref="A1:T20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Filter_Type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Tab_ID</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Insight_1</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Insight_2</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Insight_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TODAY</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>overview</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Market conditions are currently stable.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>No high-priority competitor moves detected in this timeframe.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Continue tracking standard sector intelligence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TODAY</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>growth-marketing</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>No competitor partnerships or alliances reported.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Venture funding and capital movements are currently quiet.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Monitor standard press channels for upcoming deals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TODAY</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>product-strategy</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>No competitor product launches or API releases cataloged.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Digital feature velocity remains normal.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Continue monitoring competitor release notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>7D</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>overview</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Launch a travel‑advisor‑centric API that replicates Expedia TAAP’s behind‑the‑scenes engine, allowing US travel agencies to book and manage itineraries directly through MONDEE’s platform.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Develop a white‑label travel engine for US brands, positioning MONDEE as a direct competitor to Priceline Partner Network’s white‑label offering, and begin outreach to travel agencies seeking a customizable booking solution.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Partner with Vancouver’s tourism board to create and market curated travel packages for the new Car‑Free Granville Street pedestrian zone, using MONDEE’s analytics to target travelers interested in urban experiences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>7D</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>growth-marketing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>No competitor partnerships or alliances reported.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Venture funding and capital movements are currently quiet.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Monitor standard press channels for upcoming deals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>7D</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>product-strategy</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Develop and launch a proprietary behind‑the‑scenes travel advisor engine that integrates with our existing platform, offering real‑time inventory, dynamic pricing, and a dedicated API for US travel advisors. Include a sandbox environment and partner onboarding program to accelerate adoption.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Introduce a white‑label travel engine solution similar to Priceline Partner Network, enabling travel agencies to brand our booking engine while accessing our inventory and revenue‑management tools. Offer a revenue‑share model and co‑marketing support to attract agencies.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Leverage the new back‑office API and tools announced by Expedia to build a data‑driven analytics dashboard for advisors, highlighting market trends and inventory gaps, positioning MONDEE as the data partner of choice. Pilot the dashboard with a select group of advisors to gather feedback and iterate quickly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>30D</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>overview</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Develop a back‑office API suite for travel advisors that offers real‑time inventory and dynamic pricing, directly addressing Expedia TAAP’s new tools and positioning MONDEE as the preferred platform for agency efficiency.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Launch a Vancouver‑centric travel package that highlights the new car‑free Granville Street zone, partnering with local tourism boards to capture the growing demand for sustainable urban travel experiences.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Create a white‑label travel engine tailored for boutique agencies, leveraging insights from Priceline Partner Network’s model to provide a flexible, cost‑effective alternative to Booking Holdings’ offering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>30D</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>growth-marketing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>No competitor partnerships or alliances reported.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Venture funding and capital movements are currently quiet.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Monitor standard press channels for upcoming deals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>30D</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>product-strategy</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Develop and release a back‑office API suite for travel advisors, mirroring Expedia TAAP’s new tools, to enable agencies to manage bookings and operations directly within MONDEE’s platform.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Launch a dedicated advisor‑efficiency module that automates booking reference generation and workflow management, positioning MONDEE as the most agent‑friendly platform in the market.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Introduce a white‑label travel engine similar to Priceline Partner Network, allowing partners to embed MONDEE’s inventory and booking capabilities under their own brand, thereby expanding our distribution network.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>overview</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Launch a dedicated back‑office API suite for travel advisors, mirroring Expedia TAAP’s new tools, and pilot it with our top 10 agency partners to secure early adoption and gather feedback for rapid iteration. This will position MONDEE as the preferred tech partner for agencies seeking streamlined booking and reference management.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Collaborate with Vancouver’s city council to develop a digital promotion package for the new car‑free Granville Street zone, integrating real‑time event data into our platform to drive bookings for local attractions. This partnership will enhance our visibility in the urban travel market and create a unique selling point against competitors.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Introduce a white‑label travel engine similar to Priceline Partner Network, offering agencies a customizable booking platform that can be branded and integrated into their own websites, and launch a targeted marketing campaign to agencies in the US and Canada. This will allow us to capture agency revenue streams while leveraging our existing technology stack.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>growth-marketing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>No competitor partnerships or alliances reported.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Venture funding and capital movements are currently quiet.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Monitor standard press channels for upcoming deals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>product-strategy</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Develop and launch a dedicated back‑office API suite for travel agencies, mirroring Expedia TAAP’s new tools, and beta‑test it with a select group of high‑volume advisors to gather feedback before a full rollout. This will position MONDEE as the go‑to platform for agency efficiency and enable early adoption by key partners.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Introduce a white‑label travel engine similar to Priceline Partner Network, allowing agencies to brand MONDEE’s booking infrastructure, and market it as a turnkey solution for agencies seeking to expand their product offerings.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Launch a rewards program for agencies that use MONDEE’s API, offering tiered incentives for volume and engagement, to compete with Expedia TAAP’s rewards and drive loyalty.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>